<commit_message>
chore(weekly-sync): auto-pull through 2026-06-21
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week25.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week25.xlsx
@@ -1322,10 +1322,10 @@
         <v>77503</v>
       </c>
       <c r="G32" t="n">
-        <v>67728.11</v>
+        <v>69973.03</v>
       </c>
       <c r="H32" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33">
@@ -1434,10 +1434,10 @@
         <v>1701</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>1439.83</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -2498,10 +2498,10 @@
         <v>105674</v>
       </c>
       <c r="G74" t="n">
-        <v>93138.97</v>
+        <v>85088.97</v>
       </c>
       <c r="H74" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="75">
@@ -2977,7 +2977,7 @@
         <v>12709.32</v>
       </c>
       <c r="H91" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="92">
@@ -12578,10 +12578,10 @@
         <v>931242</v>
       </c>
       <c r="G41" t="n">
-        <v>35594.92</v>
+        <v>27922.88</v>
       </c>
       <c r="H41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42">

</xml_diff>

<commit_message>
chore(weekly-sync): auto-pull through 2026-06-22
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week25.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week25.xlsx
@@ -968,190 +968,190 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Audio Array-B078WNW4YW-TONOR Wireless -SP-KT-Exact/Phrase</t>
+          <t>Audio Array-Audio Mixer-SP-KT-Exact</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>B078WNW4YW</t>
+          <t>B0G53H49BS</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>482.28</v>
+        <v>2863.99</v>
       </c>
       <c r="E20" t="n">
-        <v>34</v>
+        <v>302</v>
       </c>
       <c r="F20" t="n">
-        <v>5780</v>
+        <v>24578</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>19842.37</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Audio Array-B07GVGMW59-Tonor G11-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-Audio Mixer-SP-KT-Exact</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>B07GVGMW59</t>
+          <t>B0G53M9258</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>364.77</v>
+        <v>496.29</v>
       </c>
       <c r="E21" t="n">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="F21" t="n">
-        <v>6023</v>
+        <v>6267</v>
       </c>
       <c r="G21" t="n">
-        <v>2287.29</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Audio Array-B07GVGMW59-Tonor G11-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-Audio Mixer-SP-KT-Exact</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>B0BVHZ5MKZ</t>
+          <t>B0GCP1J2HC</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>32.81999999999999</v>
+        <v>658.6999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>110</v>
       </c>
       <c r="F22" t="n">
-        <v>771</v>
+        <v>18197</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>7033.05</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Audio Array-B07WLWN2ZT-Tonor TC 777-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-Audio Mixer-SP-KT-Exact</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>B07WLWN2ZT</t>
+          <t>B0GN2LHJY4</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>91.22999999999999</v>
+        <v>523.9400000000001</v>
       </c>
       <c r="E23" t="n">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="F23" t="n">
-        <v>2026</v>
+        <v>11961</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>8050</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Audio Array-B07WLWN2ZT-Tonor TC 777-SP-PT</t>
+          <t>Audio Array-B078WNW4YW-TONOR Wireless -SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>B07WLWN2ZT</t>
+          <t>B078WNW4YW</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>195.42</v>
+        <v>482.28</v>
       </c>
       <c r="E24" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="F24" t="n">
-        <v>2858</v>
+        <v>5780</v>
       </c>
       <c r="G24" t="n">
-        <v>2372.03</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser -SP-PT</t>
+          <t>Audio Array-B07GVGMW59-Tonor G11-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B07GVGMW59</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>3824.42</v>
+        <v>364.77</v>
       </c>
       <c r="E25" t="n">
-        <v>235</v>
+        <v>51</v>
       </c>
       <c r="F25" t="n">
-        <v>24301</v>
+        <v>6023</v>
       </c>
       <c r="G25" t="n">
-        <v>19230.54</v>
+        <v>2287.29</v>
       </c>
       <c r="H25" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP -KT-Exact</t>
+          <t>Audio Array-B07GVGMW59-Tonor G11-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B0BVHZ5MKZ</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>250.6</v>
+        <v>32.81999999999999</v>
       </c>
       <c r="E26" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
-        <v>1198</v>
+        <v>771</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -1164,63 +1164,63 @@
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP -KT-Phrase</t>
+          <t>Audio Array-B07WLWN2ZT-Tonor TC 777-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B07WLWN2ZT</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1478.7</v>
+        <v>91.22999999999999</v>
       </c>
       <c r="E27" t="n">
-        <v>78</v>
+        <v>18</v>
       </c>
       <c r="F27" t="n">
-        <v>14149</v>
+        <v>2026</v>
       </c>
       <c r="G27" t="n">
-        <v>2244.92</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP-KT-EXACT</t>
+          <t>Audio Array-B07WLWN2ZT-Tonor TC 777-SP-PT</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>B0B4DPX2J2</t>
+          <t>B07WLWN2ZT</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4188.42</v>
+        <v>195.42</v>
       </c>
       <c r="E28" t="n">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="F28" t="n">
-        <v>15482</v>
+        <v>2858</v>
       </c>
       <c r="G28" t="n">
-        <v>14105.11</v>
+        <v>2372.03</v>
       </c>
       <c r="H28" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP-KT-Exact</t>
+          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser -SP-PT</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1229,26 +1229,26 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1216.72</v>
+        <v>3824.42</v>
       </c>
       <c r="E29" t="n">
-        <v>44</v>
+        <v>235</v>
       </c>
       <c r="F29" t="n">
-        <v>3742</v>
+        <v>24301</v>
       </c>
       <c r="G29" t="n">
-        <v>2244.92</v>
+        <v>19230.54</v>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP-KT-Exact/Phrase-Branded</t>
+          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP -KT-Exact</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1257,26 +1257,26 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2742.13</v>
+        <v>250.6</v>
       </c>
       <c r="E30" t="n">
-        <v>246</v>
+        <v>15</v>
       </c>
       <c r="F30" t="n">
-        <v>21955</v>
+        <v>1198</v>
       </c>
       <c r="G30" t="n">
-        <v>43558.16</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP-PT</t>
+          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP -KT-Phrase</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1285,26 +1285,26 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1272.28</v>
+        <v>1478.7</v>
       </c>
       <c r="E31" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="F31" t="n">
-        <v>8054</v>
+        <v>14149</v>
       </c>
       <c r="G31" t="n">
-        <v>11437.3</v>
+        <v>2244.92</v>
       </c>
       <c r="H31" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4DPX2J2-Condenser AM C1 -SP-KT-Broad</t>
+          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP-KT-EXACT</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1313,26 +1313,26 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>17432.19</v>
+        <v>4188.42</v>
       </c>
       <c r="E32" t="n">
-        <v>1208</v>
+        <v>193</v>
       </c>
       <c r="F32" t="n">
-        <v>77503</v>
+        <v>15482</v>
       </c>
       <c r="G32" t="n">
-        <v>69973.03</v>
+        <v>14105.11</v>
       </c>
       <c r="H32" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4DPX2J2-Condenser AM C1-SP -KT-Broad</t>
+          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP-KT-Exact</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1341,181 +1341,181 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>274.83</v>
+        <v>1216.72</v>
       </c>
       <c r="E33" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="F33" t="n">
-        <v>1231</v>
+        <v>3742</v>
       </c>
       <c r="G33" t="n">
-        <v>13131.37</v>
+        <v>2244.92</v>
       </c>
       <c r="H33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4G19R58-AM C2 Condenser-SP -KT-Exact/Phrase</t>
+          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP-KT-Exact/Phrase-Branded</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>B0B4G19R58</t>
+          <t>B0B4DPX2J2</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1267.33</v>
+        <v>2742.13</v>
       </c>
       <c r="E34" t="n">
-        <v>70</v>
+        <v>246</v>
       </c>
       <c r="F34" t="n">
-        <v>17538</v>
+        <v>21955</v>
       </c>
       <c r="G34" t="n">
-        <v>5464.42</v>
+        <v>45803.08</v>
       </c>
       <c r="H34" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4G1PXWV-Condenser-SP-PT</t>
+          <t>Audio Array-B0B4DPX2J2-AM C1 Condenser-SP-PT</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>B0B4G1PXWV</t>
+          <t>B0B4DPX2J2</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>1272.28</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>8054</v>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>11437.3</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4G7VWXD-AA 04 Metal -SP-PT</t>
+          <t>Audio Array-B0B4DPX2J2-Condenser AM C1 -SP-KT-Broad</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>B0B4G7VWXD</t>
+          <t>B0B4DPX2J2</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>336.33</v>
+        <v>17432.19</v>
       </c>
       <c r="E36" t="n">
-        <v>21</v>
+        <v>1208</v>
       </c>
       <c r="F36" t="n">
-        <v>1701</v>
+        <v>77503</v>
       </c>
       <c r="G36" t="n">
-        <v>1439.83</v>
+        <v>69973.03</v>
       </c>
       <c r="H36" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4G7VWXD-AA 04 Metal-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-B0B4DPX2J2-Condenser AM C1-SP -KT-Broad</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>B0B4G7VWXD</t>
+          <t>B0B4DPX2J2</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>621.26</v>
+        <v>274.83</v>
       </c>
       <c r="E37" t="n">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="F37" t="n">
-        <v>6056</v>
+        <v>1231</v>
       </c>
       <c r="G37" t="n">
-        <v>8638.98</v>
+        <v>13131.37</v>
       </c>
       <c r="H37" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4G8PH2P/ B0CF5R3V95 -Microphone Stand-SP CT</t>
+          <t>Audio Array-B0B4G19R58-AM C2 Condenser-SP -KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>B0B4G8PH2P</t>
+          <t>B0B4G19R58</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>1267.33</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F38" t="n">
-        <v>135</v>
+        <v>17538</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>5464.42</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4G8PH2P/ B0CF5R3V95 -Microphone Stand-SP CT</t>
+          <t>Audio Array-B0B4G1PXWV-Condenser-SP-PT</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>B0CF5R3V95</t>
+          <t>B0B4G1PXWV</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>8.24</v>
+        <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>942</v>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -1528,203 +1528,203 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Audio Array-B0B4KC7VBM-AM C5 Conference-SP-PT</t>
+          <t>Audio Array-B0B4G7VWXD-AA 04 Metal -SP-PT</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>B0B4KC7VBM</t>
+          <t>B0B4G7VWXD</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>316.8</v>
+        <v>336.33</v>
       </c>
       <c r="E40" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F40" t="n">
-        <v>729</v>
+        <v>1701</v>
       </c>
       <c r="G40" t="n">
-        <v>5972.040000000001</v>
+        <v>1439.83</v>
       </c>
       <c r="H40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Audio Array-B0BLKBJ5HN-AM K1 Instrument-SP-PT</t>
+          <t>Audio Array-B0B4G7VWXD-AA 04 Metal-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>B0BLKBJ5HN</t>
+          <t>B0B4G7VWXD</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>4</v>
+        <v>621.26</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>66</v>
       </c>
       <c r="F41" t="n">
-        <v>19</v>
+        <v>6056</v>
       </c>
       <c r="G41" t="n">
-        <v>7880.51</v>
+        <v>8638.98</v>
       </c>
       <c r="H41" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLWW72Y-AM C28 Microphone-SP-PT</t>
+          <t>Audio Array-B0B4G8PH2P/ B0CF5R3V95 -Microphone Stand-SP CT</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>B0BPLWW72Y</t>
+          <t>B0B4G8PH2P</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2219.82</v>
+        <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>148</v>
+        <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>19002</v>
+        <v>135</v>
       </c>
       <c r="G42" t="n">
-        <v>5420.32</v>
+        <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface -SP -CT</t>
+          <t>Audio Array-B0B4G8PH2P/ B0CF5R3V95 -Microphone Stand-SP CT</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>B0BPLZ5CGV</t>
+          <t>B0CF5R3V95</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>242.33</v>
+        <v>8.24</v>
       </c>
       <c r="E43" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="F43" t="n">
-        <v>4510</v>
+        <v>942</v>
       </c>
       <c r="G43" t="n">
-        <v>8133.9</v>
+        <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface -SP-AT</t>
+          <t>Audio Array-B0B4KC7VBM-AM C5 Conference-SP-PT</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>B0BPLZ5CGV</t>
+          <t>B0B4KC7VBM</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>316.8</v>
       </c>
       <c r="E44" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>729</v>
       </c>
       <c r="G44" t="n">
-        <v>0</v>
+        <v>5972.040000000001</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface -SP-PT</t>
+          <t>Audio Array-B0BLKBJ5HN-AM K1 Instrument-SP-PT</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>B0BPLZ5CGV</t>
+          <t>B0BLKBJ5HN</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1096.67</v>
+        <v>4</v>
       </c>
       <c r="E45" t="n">
-        <v>67</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>5346</v>
+        <v>19</v>
       </c>
       <c r="G45" t="n">
-        <v>8133.9</v>
+        <v>7880.51</v>
       </c>
       <c r="H45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface-SP-KT-EXACT</t>
+          <t>Audio Array-B0BPLWW72Y-AM C28 Microphone-SP-PT</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>B0BPLZ5CGV</t>
+          <t>B0BPLWW72Y</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>212.55</v>
+        <v>2219.82</v>
       </c>
       <c r="E46" t="n">
-        <v>8</v>
+        <v>148</v>
       </c>
       <c r="F46" t="n">
-        <v>471</v>
+        <v>19002</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>5420.32</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface-SP-KT-Exact</t>
+          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface -SP -CT</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1733,26 +1733,26 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>3271.29</v>
+        <v>242.33</v>
       </c>
       <c r="E47" t="n">
-        <v>366</v>
+        <v>31</v>
       </c>
       <c r="F47" t="n">
-        <v>62985</v>
+        <v>4510</v>
       </c>
       <c r="G47" t="n">
-        <v>16690.68</v>
+        <v>8133.9</v>
       </c>
       <c r="H47" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface-SP-KT-Exact/Phrase-Branded</t>
+          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface -SP-AT</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1761,26 +1761,26 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>4292.16</v>
+        <v>0</v>
       </c>
       <c r="E48" t="n">
-        <v>319</v>
+        <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>44439</v>
+        <v>0</v>
       </c>
       <c r="G48" t="n">
-        <v>60542.36</v>
+        <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface-SP-PT</t>
+          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface -SP-PT</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1789,26 +1789,26 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>1096.67</v>
       </c>
       <c r="E49" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
+        <v>5346</v>
       </c>
       <c r="G49" t="n">
-        <v>0</v>
+        <v>8133.9</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-Audio Interface AI 04 -SP-KT-Broad_Branded</t>
+          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface-SP-KT-EXACT</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1817,26 +1817,26 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>7928.98</v>
+        <v>212.55</v>
       </c>
       <c r="E50" t="n">
-        <v>1047</v>
+        <v>8</v>
       </c>
       <c r="F50" t="n">
-        <v>124346</v>
+        <v>471</v>
       </c>
       <c r="G50" t="n">
-        <v>75534.75</v>
+        <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-Audio Interface-SP-KT-Exact</t>
+          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface-SP-KT-Exact</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1845,16 +1845,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2273.07</v>
+        <v>3271.29</v>
       </c>
       <c r="E51" t="n">
-        <v>188</v>
+        <v>366</v>
       </c>
       <c r="F51" t="n">
-        <v>12572</v>
+        <v>62985</v>
       </c>
       <c r="G51" t="n">
-        <v>16775.41</v>
+        <v>16690.68</v>
       </c>
       <c r="H51" t="n">
         <v>5</v>
@@ -1864,7 +1864,7 @@
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-Interface AI 04-SP -KT</t>
+          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface-SP-KT-Exact/Phrase-Branded</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1873,26 +1873,26 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>21.21</v>
+        <v>4292.16</v>
       </c>
       <c r="E52" t="n">
-        <v>5</v>
+        <v>319</v>
       </c>
       <c r="F52" t="n">
-        <v>372</v>
+        <v>44439</v>
       </c>
       <c r="G52" t="n">
-        <v>4066.95</v>
+        <v>60542.36</v>
       </c>
       <c r="H52" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Audio Array-B0BPLZ5CGV-Interface AI 04-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-B0BPLZ5CGV-AI 04 Interface-SP-PT</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1901,181 +1901,181 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>16852.87</v>
+        <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>1099</v>
+        <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>182991</v>
+        <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>71935.60000000001</v>
+        <v>0</v>
       </c>
       <c r="H53" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Audio Array-B0BRKFP94K-TONOR TD510-SP-PT</t>
+          <t>Audio Array-B0BPLZ5CGV-Audio Interface AI 04 -SP-KT-Broad_Branded</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>B0BRKFP94K</t>
+          <t>B0BPLZ5CGV</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>7928.98</v>
       </c>
       <c r="E54" t="n">
-        <v>0</v>
+        <v>1047</v>
       </c>
       <c r="F54" t="n">
-        <v>19</v>
+        <v>124346</v>
       </c>
       <c r="G54" t="n">
-        <v>0</v>
+        <v>64943.22</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Audio Array-B0BYHHSLPC-Tonor TC 777pro-SP-PT</t>
+          <t>Audio Array-B0BPLZ5CGV-Audio Interface-SP-KT-Exact</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>B0BYHHSLPC</t>
+          <t>B0BPLZ5CGV</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>2273.07</v>
       </c>
       <c r="E55" t="n">
-        <v>0</v>
+        <v>188</v>
       </c>
       <c r="F55" t="n">
-        <v>78</v>
+        <v>12572</v>
       </c>
       <c r="G55" t="n">
-        <v>0</v>
+        <v>16775.41</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Audio Array-B0CF5TCQKL-AA 21 Desktop-SP -KT-Exact/Phrase</t>
+          <t>Audio Array-B0BPLZ5CGV-Interface AI 04-SP -KT</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>B0CF5TCQKL</t>
+          <t>B0BPLZ5CGV</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>7622.07</v>
+        <v>21.21</v>
       </c>
       <c r="E56" t="n">
-        <v>272</v>
+        <v>5</v>
       </c>
       <c r="F56" t="n">
-        <v>22259</v>
+        <v>372</v>
       </c>
       <c r="G56" t="n">
-        <v>19264.4</v>
+        <v>4066.95</v>
       </c>
       <c r="H56" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Audio Array-B0CF5TCQKL-AA 21 Desktop-SP-PT</t>
+          <t>Audio Array-B0BPLZ5CGV-Interface AI 04-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>B0CF5TCQKL</t>
+          <t>B0BPLZ5CGV</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1770.62</v>
+        <v>16852.87</v>
       </c>
       <c r="E57" t="n">
-        <v>130</v>
+        <v>1099</v>
       </c>
       <c r="F57" t="n">
-        <v>6050</v>
+        <v>182990</v>
       </c>
       <c r="G57" t="n">
-        <v>12877.96</v>
+        <v>71935.60000000001</v>
       </c>
       <c r="H57" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Audio Array-B0CH4RNWJX-AM C43-SP-KT -Exact/Phrase</t>
+          <t>Audio Array-B0BRKFP94K-TONOR TD510-SP-PT</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>B0CH4RNWJX</t>
+          <t>B0BRKFP94K</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>4122.01</v>
+        <v>0</v>
       </c>
       <c r="E58" t="n">
-        <v>201</v>
+        <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>35269</v>
+        <v>19</v>
       </c>
       <c r="G58" t="n">
-        <v>15925.44</v>
+        <v>0</v>
       </c>
       <c r="H58" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Audio Array-B0CH4RNWJX-AM C43-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-B0BYHHSLPC-Tonor TC 777pro-SP-PT</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>B0CH4RNWJX</t>
+          <t>B0BYHHSLPC</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>897.9400000000001</v>
+        <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>12464</v>
+        <v>78</v>
       </c>
       <c r="G59" t="n">
         <v>0</v>
@@ -2088,147 +2088,147 @@
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Audio Array-B0CH4RNWJX-AM C43-SP-PT</t>
+          <t>Audio Array-B0CF5TCQKL-AA 21 Desktop-SP -KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>B0CH4RNWJX</t>
+          <t>B0CF5TCQKL</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>155.87</v>
+        <v>7622.07</v>
       </c>
       <c r="E60" t="n">
-        <v>24</v>
+        <v>272</v>
       </c>
       <c r="F60" t="n">
-        <v>3451</v>
+        <v>22259</v>
       </c>
       <c r="G60" t="n">
-        <v>3515.26</v>
+        <v>19264.4</v>
       </c>
       <c r="H60" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Audio Array-B0CKHVHVQ1-AM W45 Microphone-SP-CT</t>
+          <t>Audio Array-B0CF5TCQKL-AA 21 Desktop-SP-PT</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>B0CKHVHVQ1</t>
+          <t>B0CF5TCQKL</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>2681.22</v>
+        <v>1770.62</v>
       </c>
       <c r="E61" t="n">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="F61" t="n">
-        <v>19199</v>
+        <v>6050</v>
       </c>
       <c r="G61" t="n">
-        <v>13217.79</v>
+        <v>12877.96</v>
       </c>
       <c r="H61" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Audio Array-B0CKHVHVQ1-AM W45 Microphone-SP-KT</t>
+          <t>Audio Array-B0CH4RNWJX-AM C43-SP-KT -Exact/Phrase</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>B0CKHVHVQ1</t>
+          <t>B0CH4RNWJX</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>996.54</v>
+        <v>4122.01</v>
       </c>
       <c r="E62" t="n">
-        <v>135</v>
+        <v>201</v>
       </c>
       <c r="F62" t="n">
-        <v>17364</v>
+        <v>35269</v>
       </c>
       <c r="G62" t="n">
-        <v>17623.73</v>
+        <v>15925.44</v>
       </c>
       <c r="H62" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless -SP-KT-Exact/Phrase</t>
+          <t>Audio Array-B0CH4RNWJX-AM C43-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>B0CKHVHVQ1</t>
+          <t>B0CH4RNWJX</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1699.19</v>
+        <v>897.9400000000001</v>
       </c>
       <c r="E63" t="n">
-        <v>103</v>
+        <v>44</v>
       </c>
       <c r="F63" t="n">
-        <v>8431</v>
+        <v>12464</v>
       </c>
       <c r="G63" t="n">
-        <v>8811.860000000001</v>
+        <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-B0CH4RNWJX-AM C43-SP-PT</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>B0CKHVHVQ1</t>
+          <t>B0CH4RNWJX</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>616.48</v>
+        <v>155.87</v>
       </c>
       <c r="E64" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="F64" t="n">
-        <v>2564</v>
+        <v>3451</v>
       </c>
       <c r="G64" t="n">
-        <v>8811.860000000001</v>
+        <v>3515.26</v>
       </c>
       <c r="H64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SP-PT</t>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Microphone-SP-CT</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2237,13 +2237,13 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>1034.75</v>
+        <v>2681.22</v>
       </c>
       <c r="E65" t="n">
-        <v>68</v>
+        <v>123</v>
       </c>
       <c r="F65" t="n">
-        <v>4008</v>
+        <v>19199</v>
       </c>
       <c r="G65" t="n">
         <v>13217.79</v>
@@ -2256,7 +2256,7 @@
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SP-PT (2)</t>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Microphone-SP-KT</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2265,128 +2265,128 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>274.77</v>
+        <v>996.54</v>
       </c>
       <c r="E66" t="n">
-        <v>24</v>
+        <v>135</v>
       </c>
       <c r="F66" t="n">
-        <v>2864</v>
+        <v>17364</v>
       </c>
       <c r="G66" t="n">
-        <v>4405.93</v>
+        <v>17623.73</v>
       </c>
       <c r="H66" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Audio Array-B0CM6NTWBP-AI 10 Condenser-SP-CT</t>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless -SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>B0CM6NTWBP</t>
+          <t>B0CKHVHVQ1</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>391.74</v>
+        <v>1699.19</v>
       </c>
       <c r="E67" t="n">
-        <v>64</v>
+        <v>103</v>
       </c>
       <c r="F67" t="n">
-        <v>5568</v>
+        <v>8431</v>
       </c>
       <c r="G67" t="n">
-        <v>8472.030000000001</v>
+        <v>8811.860000000001</v>
       </c>
       <c r="H67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Audio Array-B0CM6NTWBP-AI 10 Soundcard-SP-Auto</t>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>B0CM6NTWBP</t>
+          <t>B0CKHVHVQ1</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>1749.48</v>
+        <v>616.48</v>
       </c>
       <c r="E68" t="n">
-        <v>418</v>
+        <v>36</v>
       </c>
       <c r="F68" t="n">
-        <v>66547</v>
+        <v>2564</v>
       </c>
       <c r="G68" t="n">
-        <v>940.6799999999999</v>
+        <v>8811.860000000001</v>
       </c>
       <c r="H68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr"/>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Audio Array-B0CM6NTWBP-AI 10 Soundcard-SP-KT-Broad</t>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SP-PT</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>B0CM6NTWBP</t>
+          <t>B0CKHVHVQ1</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>32.93</v>
+        <v>1034.75</v>
       </c>
       <c r="E69" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="F69" t="n">
-        <v>877</v>
+        <v>4008</v>
       </c>
       <c r="G69" t="n">
-        <v>0</v>
+        <v>13217.79</v>
       </c>
       <c r="H69" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Audio Array-B0CM6WH4ZT-AI 12 Soundcard-SP-PT</t>
+          <t>Audio Array-B0CKHVHVQ1-AM W45 Wireless-SP-PT (2)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>B0CM6WH4ZT</t>
+          <t>B0CKHVHVQ1</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>739.91</v>
+        <v>274.77</v>
       </c>
       <c r="E70" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="F70" t="n">
-        <v>6640</v>
+        <v>2864</v>
       </c>
       <c r="G70" t="n">
-        <v>1185.59</v>
+        <v>4405.93</v>
       </c>
       <c r="H70" t="n">
         <v>1</v>
@@ -2396,25 +2396,25 @@
       <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Audio Array-B0CM9HYVDM-AM W18 Wireless Karaoke-SP-KT-Exact</t>
+          <t>Audio Array-B0CM6NTWBP-AI 10 Condenser-SP-CT</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>B0CM9HYVDM</t>
+          <t>B0CM6NTWBP</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>758.4400000000001</v>
+        <v>391.74</v>
       </c>
       <c r="E71" t="n">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="F71" t="n">
-        <v>13929</v>
+        <v>5568</v>
       </c>
       <c r="G71" t="n">
-        <v>3022.89</v>
+        <v>8472.030000000001</v>
       </c>
       <c r="H71" t="n">
         <v>3</v>
@@ -2424,442 +2424,442 @@
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Audio Array-B0DN6MNS1X-Dynamic AM C11 Pro-SP-PT</t>
+          <t>Audio Array-B0CM6NTWBP-AI 10 Soundcard-SP-Auto</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>B0DN6MNS1X</t>
+          <t>B0CM6NTWBP</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>51.38</v>
+        <v>1749.48</v>
       </c>
       <c r="E72" t="n">
-        <v>3</v>
+        <v>418</v>
       </c>
       <c r="F72" t="n">
-        <v>718</v>
+        <v>66547</v>
       </c>
       <c r="G72" t="n">
-        <v>0</v>
+        <v>940.6799999999999</v>
       </c>
       <c r="H72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Audio Array-B0DT6T6N6B-AA 26 Tabletop-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-B0CM6NTWBP-AI 10 Soundcard-SP-KT-Broad</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>B0DT6T6N6B</t>
+          <t>B0CM6NTWBP</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>1281.91</v>
+        <v>32.93</v>
       </c>
       <c r="E73" t="n">
-        <v>150</v>
+        <v>8</v>
       </c>
       <c r="F73" t="n">
-        <v>10912</v>
+        <v>877</v>
       </c>
       <c r="G73" t="n">
-        <v>2543.24</v>
+        <v>0</v>
       </c>
       <c r="H73" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Audio Array-B0DXFPM4N2-AM S1 Studio-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-B0CM6WH4ZT-AI 12 Soundcard-SP-PT</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>B0DXFPM4N2</t>
+          <t>B0CM6WH4ZT</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>11905.46</v>
+        <v>739.91</v>
       </c>
       <c r="E74" t="n">
-        <v>814</v>
+        <v>83</v>
       </c>
       <c r="F74" t="n">
-        <v>105674</v>
+        <v>6640</v>
       </c>
       <c r="G74" t="n">
-        <v>85088.97</v>
+        <v>1185.59</v>
       </c>
       <c r="H74" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Audio Array-B0FFB6YJM1-Sb 01 Soundbar-SP-Auto</t>
+          <t>Audio Array-B0CM9HYVDM-AM W18 Wireless Karaoke-SP-KT-Exact</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>B0FFB6YJM1</t>
+          <t>B0CM9HYVDM</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>3916.29</v>
+        <v>758.4400000000001</v>
       </c>
       <c r="E75" t="n">
-        <v>832</v>
+        <v>51</v>
       </c>
       <c r="F75" t="n">
-        <v>172535</v>
+        <v>13929</v>
       </c>
       <c r="G75" t="n">
-        <v>13251.67</v>
+        <v>3022.89</v>
       </c>
       <c r="H75" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Audio Array-B0FG88HVQ8-AH-50 DJ Headphone-SP-PT</t>
+          <t>Audio Array-B0DN6MNS1X-Dynamic AM C11 Pro-SP-PT</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>B0FG88HVQ8</t>
+          <t>B0DN6MNS1X</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>3287.59</v>
+        <v>51.38</v>
       </c>
       <c r="E76" t="n">
-        <v>212</v>
+        <v>3</v>
       </c>
       <c r="F76" t="n">
-        <v>9230</v>
+        <v>718</v>
       </c>
       <c r="G76" t="n">
-        <v>16940.7</v>
+        <v>0</v>
       </c>
       <c r="H76" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Audio Array-B0FG88HVQ8-DJ Headphone-SP-CT</t>
+          <t>Audio Array-B0DT6T6N6B-AA 26 Tabletop-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>B0FG88HVQ8</t>
+          <t>B0DT6T6N6B</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1607.02</v>
+        <v>1281.91</v>
       </c>
       <c r="E77" t="n">
         <v>150</v>
       </c>
       <c r="F77" t="n">
-        <v>15154</v>
+        <v>10912</v>
       </c>
       <c r="G77" t="n">
-        <v>13552.56</v>
+        <v>2543.24</v>
       </c>
       <c r="H77" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Audio Array-B0FG88HVQ8-DJ Headphone-SP-KT-Broad</t>
+          <t>Audio Array-B0DXFPM4N2-AM S1 Studio-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>B0FG88HVQ8</t>
+          <t>B0DXFPM4N2</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>248.54</v>
+        <v>11905.46</v>
       </c>
       <c r="E78" t="n">
-        <v>45</v>
+        <v>814</v>
       </c>
       <c r="F78" t="n">
-        <v>4226</v>
+        <v>105674</v>
       </c>
       <c r="G78" t="n">
-        <v>1694.07</v>
+        <v>85088.97</v>
       </c>
       <c r="H78" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Audio Array-B0FG88HVQ8-DJ Headphone-SP-KT-Exact</t>
+          <t>Audio Array-B0FFB6YJM1-Sb 01 Soundbar-SP-Auto</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>B0FG88HVQ8</t>
+          <t>B0FFB6YJM1</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>2508.27</v>
+        <v>3916.29</v>
       </c>
       <c r="E79" t="n">
-        <v>107</v>
+        <v>832</v>
       </c>
       <c r="F79" t="n">
-        <v>12031</v>
+        <v>172535</v>
       </c>
       <c r="G79" t="n">
-        <v>5082.209999999999</v>
+        <v>13251.67</v>
       </c>
       <c r="H79" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Audio Array-B0G39ZHDYP-Voice Amplifier-SP-CT/PT</t>
+          <t>Audio Array-B0FG88HVQ8-AH-50 DJ Headphone-SP-PT</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>B0G39ZHDYP</t>
+          <t>B0FG88HVQ8</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>4688.62</v>
+        <v>3287.59</v>
       </c>
       <c r="E80" t="n">
-        <v>354</v>
+        <v>212</v>
       </c>
       <c r="F80" t="n">
-        <v>54491</v>
+        <v>9230</v>
       </c>
       <c r="G80" t="n">
-        <v>16005.06</v>
+        <v>17405.95</v>
       </c>
       <c r="H80" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Audio Array-B0G39ZHDYP-Voice Amplifier-SP-KT-BM</t>
+          <t>Audio Array-B0FG88HVQ8-DJ Headphone-SP-CT</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>B0G39ZHDYP</t>
+          <t>B0FG88HVQ8</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>2644.53</v>
+        <v>1607.02</v>
       </c>
       <c r="E81" t="n">
-        <v>227</v>
+        <v>150</v>
       </c>
       <c r="F81" t="n">
-        <v>55146</v>
+        <v>15154</v>
       </c>
       <c r="G81" t="n">
-        <v>4064.4</v>
+        <v>13552.56</v>
       </c>
       <c r="H81" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Audio Array-B0G4DNF8RZ-AM C48 Dynamic -SP-Auto</t>
+          <t>Audio Array-B0FG88HVQ8-DJ Headphone-SP-KT-Broad</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>B0G4DNF8RZ</t>
+          <t>B0FG88HVQ8</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>970.42</v>
+        <v>248.54</v>
       </c>
       <c r="E82" t="n">
-        <v>123</v>
+        <v>45</v>
       </c>
       <c r="F82" t="n">
-        <v>24938</v>
+        <v>4226</v>
       </c>
       <c r="G82" t="n">
-        <v>5591.52</v>
+        <v>1694.07</v>
       </c>
       <c r="H82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Audio Array-B0G4DNF8RZ-Dynamic AM C48-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-B0FG88HVQ8-DJ Headphone-SP-KT-Exact</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>B0G4DNF8RZ</t>
+          <t>B0FG88HVQ8</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>144.47</v>
+        <v>2508.27</v>
       </c>
       <c r="E83" t="n">
-        <v>16</v>
+        <v>107</v>
       </c>
       <c r="F83" t="n">
-        <v>2127</v>
+        <v>12031</v>
       </c>
       <c r="G83" t="n">
-        <v>0</v>
+        <v>5082.209999999999</v>
       </c>
       <c r="H83" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr"/>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Audio Array-B0G53H49BS-AI 13 Hybrid USB-SP-KT -Exact/Phrase</t>
+          <t>Audio Array-B0G39ZHDYP-Voice Amplifier-SP-CT/PT</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>B0G53H49BS</t>
+          <t>B0G39ZHDYP</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>4480.52</v>
+        <v>4688.62</v>
       </c>
       <c r="E84" t="n">
-        <v>494</v>
+        <v>354</v>
       </c>
       <c r="F84" t="n">
-        <v>56755</v>
+        <v>54489</v>
       </c>
       <c r="G84" t="n">
-        <v>14358.47</v>
+        <v>16005.06</v>
       </c>
       <c r="H84" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Audio Array-B0G53H49BS-AI 13 Hybrid USB-SP-PT</t>
+          <t>Audio Array-B0G39ZHDYP-Voice Amplifier-SP-KT-BM</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>B0G53H49BS</t>
+          <t>B0G39ZHDYP</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>6459.94</v>
+        <v>2644.53</v>
       </c>
       <c r="E85" t="n">
-        <v>524</v>
+        <v>227</v>
       </c>
       <c r="F85" t="n">
-        <v>10085</v>
+        <v>55144</v>
       </c>
       <c r="G85" t="n">
-        <v>25965.26</v>
+        <v>4064.4</v>
       </c>
       <c r="H85" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Audio Array-B0G53H49BS-AI 13 Mixer-SP-KT -Broad</t>
+          <t>Audio Array-B0G4DNF8RZ-AM C48 Dynamic -SP-Auto</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>B0G53H49BS</t>
+          <t>B0G4DNF8RZ</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>225.68</v>
+        <v>970.42</v>
       </c>
       <c r="E86" t="n">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="F86" t="n">
-        <v>5079</v>
+        <v>24937</v>
       </c>
       <c r="G86" t="n">
-        <v>0</v>
+        <v>5591.52</v>
       </c>
       <c r="H86" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr"/>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Audio Array-B0GN8RQJRG-AK 37 Velocity-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-B0G4DNF8RZ-Dynamic AM C48-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>B0GN8RQJRG</t>
+          <t>B0G4DNF8RZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0</v>
+        <v>144.47</v>
       </c>
       <c r="E87" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F87" t="n">
-        <v>0</v>
+        <v>2127</v>
       </c>
       <c r="G87" t="n">
         <v>0</v>
@@ -2872,236 +2872,236 @@
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Audio Array-B0GN97RFPR-AM S2 Studio-SP-KT-Exact/Phrase</t>
+          <t>Audio Array-B0G53H49BS-AI 13 Hybrid USB-SP-KT -Exact/Phrase</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>B0GN97RFPR</t>
+          <t>B0G53H49BS</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>12724.12</v>
+        <v>4480.52</v>
       </c>
       <c r="E88" t="n">
-        <v>1036</v>
+        <v>494</v>
       </c>
       <c r="F88" t="n">
-        <v>103196</v>
+        <v>56755</v>
       </c>
       <c r="G88" t="n">
-        <v>98942.53</v>
+        <v>14358.47</v>
       </c>
       <c r="H88" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Audio Array-B0GN97RFPR-Studio AM S2 -SP-CT</t>
+          <t>Audio Array-B0G53H49BS-AI 13 Hybrid USB-SP-PT</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>B0GN97RFPR</t>
+          <t>B0G53H49BS</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>7214.16</v>
+        <v>6459.94</v>
       </c>
       <c r="E89" t="n">
-        <v>536</v>
+        <v>524</v>
       </c>
       <c r="F89" t="n">
-        <v>22557</v>
+        <v>10085</v>
       </c>
       <c r="G89" t="n">
-        <v>58043.22</v>
+        <v>25965.26</v>
       </c>
       <c r="H89" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Audio Array-B0GN97RFPR-Studio AM S2-SP -PT</t>
+          <t>Audio Array-B0G53H49BS-AI 13 Mixer-SP-KT -Broad</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>B0GN97RFPR</t>
+          <t>B0G53H49BS</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>2569.55</v>
+        <v>225.68</v>
       </c>
       <c r="E90" t="n">
-        <v>264</v>
+        <v>60</v>
       </c>
       <c r="F90" t="n">
-        <v>17095</v>
+        <v>5079</v>
       </c>
       <c r="G90" t="n">
-        <v>19573.74</v>
+        <v>0</v>
       </c>
       <c r="H90" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr"/>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All -AK 61 Portable-SP-AT</t>
+          <t>Audio Array-B0GN8RQJRG-AK 37 Velocity-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>B0GN8MFDGZ</t>
+          <t>B0GN8RQJRG</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1061.13</v>
+        <v>0</v>
       </c>
       <c r="E91" t="n">
-        <v>288</v>
+        <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>36307</v>
+        <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>12709.32</v>
+        <v>0</v>
       </c>
       <c r="H91" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All -AK 61 Portable-SP-AT</t>
+          <t>Audio Array-B0GN97RFPR-AM S2 Studio-SP-KT-Exact/Phrase</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>B0GN8MMKY1</t>
+          <t>B0GN97RFPR</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0</v>
+        <v>12724.12</v>
       </c>
       <c r="E92" t="n">
-        <v>0</v>
+        <v>1036</v>
       </c>
       <c r="F92" t="n">
-        <v>0</v>
+        <v>103196</v>
       </c>
       <c r="G92" t="n">
-        <v>0</v>
+        <v>98942.53</v>
       </c>
       <c r="H92" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr"/>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All -AK 61 Portable-SP-AT</t>
+          <t>Audio Array-B0GN97RFPR-Studio AM S2 -SP-CT</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>B0GN8MPYPG</t>
+          <t>B0GN97RFPR</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>1191.68</v>
+        <v>7214.16</v>
       </c>
       <c r="E93" t="n">
-        <v>353</v>
+        <v>536</v>
       </c>
       <c r="F93" t="n">
-        <v>45829</v>
+        <v>22557</v>
       </c>
       <c r="G93" t="n">
-        <v>9320.34</v>
+        <v>58043.22</v>
       </c>
       <c r="H93" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr"/>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All -AK 61 Portable-SP-AT</t>
+          <t>Audio Array-B0GN97RFPR-Studio AM S2-SP -PT</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>B0GN8RQJRG</t>
+          <t>B0GN97RFPR</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0</v>
+        <v>2569.55</v>
       </c>
       <c r="E94" t="n">
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="F94" t="n">
-        <v>0</v>
+        <v>17095</v>
       </c>
       <c r="G94" t="n">
-        <v>0</v>
+        <v>19573.74</v>
       </c>
       <c r="H94" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr"/>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All-Audio Interface-SP-Brand -KT-Exact</t>
+          <t>Audio Array-Catch All -AK 61 Portable-SP-AT</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>B0CM6NTWBP</t>
+          <t>B0GN8MFDGZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0</v>
+        <v>1061.13</v>
       </c>
       <c r="E95" t="n">
-        <v>0</v>
+        <v>288</v>
       </c>
       <c r="F95" t="n">
-        <v>0</v>
+        <v>36306</v>
       </c>
       <c r="G95" t="n">
-        <v>0</v>
+        <v>12709.32</v>
       </c>
       <c r="H95" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr"/>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All-Audio Interface-SP-Brand -KT-Exact</t>
+          <t>Audio Array-Catch All -AK 61 Portable-SP-AT</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>B0CM6NVLT9</t>
+          <t>B0GN8MMKY1</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -3124,50 +3124,50 @@
       <c r="A97" t="inlineStr"/>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All-Audio Mixer-SP-KT-Exact</t>
+          <t>Audio Array-Catch All -AK 61 Portable-SP-AT</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>B0G53H49BS</t>
+          <t>B0GN8MPYPG</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>2863.99</v>
+        <v>1191.68</v>
       </c>
       <c r="E97" t="n">
-        <v>302</v>
+        <v>353</v>
       </c>
       <c r="F97" t="n">
-        <v>24578</v>
+        <v>45828</v>
       </c>
       <c r="G97" t="n">
-        <v>19842.37</v>
+        <v>9320.34</v>
       </c>
       <c r="H97" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr"/>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All-Audio Mixer-SP-KT-Exact</t>
+          <t>Audio Array-Catch All -AK 61 Portable-SP-AT</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>B0G53M9258</t>
+          <t>B0GN8RQJRG</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>496.29</v>
+        <v>0</v>
       </c>
       <c r="E98" t="n">
-        <v>89</v>
+        <v>0</v>
       </c>
       <c r="F98" t="n">
-        <v>6267</v>
+        <v>0</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -3180,56 +3180,56 @@
       <c r="A99" t="inlineStr"/>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All-Audio Mixer-SP-KT-Exact</t>
+          <t>Audio Array-Catch All-Audio Interface-SP-Brand -KT-Exact</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>B0GCP1J2HC</t>
+          <t>B0CM6NTWBP</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>658.6999999999999</v>
+        <v>0</v>
       </c>
       <c r="E99" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="F99" t="n">
-        <v>18197</v>
+        <v>0</v>
       </c>
       <c r="G99" t="n">
-        <v>7033.05</v>
+        <v>0</v>
       </c>
       <c r="H99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Audio Array-Catch All-Audio Mixer-SP-KT-Exact</t>
+          <t>Audio Array-Catch All-Audio Interface-SP-Brand -KT-Exact</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>B0GN2LHJY4</t>
+          <t>B0CM6NVLT9</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>523.9400000000001</v>
+        <v>0</v>
       </c>
       <c r="E100" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="F100" t="n">
-        <v>11961</v>
+        <v>0</v>
       </c>
       <c r="G100" t="n">
-        <v>8050</v>
+        <v>0</v>
       </c>
       <c r="H100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -4150,10 +4150,10 @@
         <v>152018</v>
       </c>
       <c r="G133" t="n">
-        <v>4532.2</v>
+        <v>7412.71</v>
       </c>
       <c r="H133" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="134">
@@ -5155,7 +5155,7 @@
         <v>10</v>
       </c>
       <c r="F169" t="n">
-        <v>2730</v>
+        <v>2729</v>
       </c>
       <c r="G169" t="n">
         <v>0</v>
@@ -5687,7 +5687,7 @@
         <v>39</v>
       </c>
       <c r="F188" t="n">
-        <v>10714</v>
+        <v>10713</v>
       </c>
       <c r="G188" t="n">
         <v>1609.32</v>
@@ -5715,7 +5715,7 @@
         <v>12</v>
       </c>
       <c r="F189" t="n">
-        <v>3643</v>
+        <v>3642</v>
       </c>
       <c r="G189" t="n">
         <v>0</v>
@@ -5855,7 +5855,7 @@
         <v>2102</v>
       </c>
       <c r="F194" t="n">
-        <v>297710</v>
+        <v>297709</v>
       </c>
       <c r="G194" t="n">
         <v>13342.37</v>
@@ -6045,13 +6045,13 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>8821.17</v>
+        <v>8820.17</v>
       </c>
       <c r="E201" t="n">
-        <v>3093</v>
+        <v>3092</v>
       </c>
       <c r="F201" t="n">
-        <v>399978</v>
+        <v>399975</v>
       </c>
       <c r="G201" t="n">
         <v>19573.74</v>
@@ -6334,10 +6334,10 @@
         <v>23079</v>
       </c>
       <c r="G211" t="n">
-        <v>19949.99</v>
+        <v>22322.02</v>
       </c>
       <c r="H211" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="212">
@@ -6680,56 +6680,56 @@
       <c r="A224" t="inlineStr"/>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Audio Array-DJ Headphones-Multi Ad Group-SP -KT-Exact</t>
+          <t>Audio Array-DJ Headphones- B0FQBXS6Y2 -SP-PT</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>B0FG88HVQ8</t>
+          <t>B0FQBWV1ST</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>2240.18</v>
+        <v>0</v>
       </c>
       <c r="E224" t="n">
-        <v>142</v>
+        <v>0</v>
       </c>
       <c r="F224" t="n">
-        <v>16664</v>
+        <v>0</v>
       </c>
       <c r="G224" t="n">
-        <v>9825.41</v>
+        <v>0</v>
       </c>
       <c r="H224" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr"/>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Audio Array-DJ Headphones-Multi Ad Group-SP -KT-Exact</t>
+          <t>Audio Array-DJ Headphones- B0FQBXS6Y2 -SP-PT</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>B0FQBTRM28</t>
+          <t>B0FQBXS6Y2</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>415.11</v>
+        <v>147.86</v>
       </c>
       <c r="E225" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F225" t="n">
-        <v>2839</v>
+        <v>966</v>
       </c>
       <c r="G225" t="n">
-        <v>0</v>
+        <v>1355.08</v>
       </c>
       <c r="H225" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="226">
@@ -6741,45 +6741,45 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>B0FQBXS6Y2</t>
+          <t>B0FG88HVQ8</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>270.91</v>
+        <v>2240.18</v>
       </c>
       <c r="E226" t="n">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="F226" t="n">
-        <v>2130</v>
+        <v>16664</v>
       </c>
       <c r="G226" t="n">
-        <v>0</v>
+        <v>9825.41</v>
       </c>
       <c r="H226" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr"/>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Audio Array-DJ Headphones-Multi Ad Groups -SP-PT</t>
+          <t>Audio Array-DJ Headphones-Multi Ad Group-SP -KT-Exact</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>B0FQBWV1ST</t>
+          <t>B0FQBTRM28</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>0</v>
+        <v>415.11</v>
       </c>
       <c r="E227" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F227" t="n">
-        <v>0</v>
+        <v>2839</v>
       </c>
       <c r="G227" t="n">
         <v>0</v>
@@ -6792,7 +6792,7 @@
       <c r="A228" t="inlineStr"/>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Audio Array-DJ Headphones-Multi Ad Groups -SP-PT</t>
+          <t>Audio Array-DJ Headphones-Multi Ad Group-SP -KT-Exact</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -6801,19 +6801,19 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>147.86</v>
+        <v>270.91</v>
       </c>
       <c r="E228" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F228" t="n">
-        <v>966</v>
+        <v>2130</v>
       </c>
       <c r="G228" t="n">
-        <v>1355.08</v>
+        <v>0</v>
       </c>
       <c r="H228" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="229">
@@ -6947,7 +6947,7 @@
         <v>77</v>
       </c>
       <c r="F233" t="n">
-        <v>14911</v>
+        <v>14907</v>
       </c>
       <c r="G233" t="n">
         <v>3302.55</v>
@@ -7227,7 +7227,7 @@
         <v>372</v>
       </c>
       <c r="F243" t="n">
-        <v>54567</v>
+        <v>54566</v>
       </c>
       <c r="G243" t="n">
         <v>13722.05</v>
@@ -7283,7 +7283,7 @@
         <v>58</v>
       </c>
       <c r="F245" t="n">
-        <v>14790</v>
+        <v>14789</v>
       </c>
       <c r="G245" t="n">
         <v>0</v>
@@ -7479,7 +7479,7 @@
         <v>114</v>
       </c>
       <c r="F252" t="n">
-        <v>16730</v>
+        <v>16726</v>
       </c>
       <c r="G252" t="n">
         <v>13597.44</v>
@@ -7647,7 +7647,7 @@
         <v>992</v>
       </c>
       <c r="F258" t="n">
-        <v>144815</v>
+        <v>144814</v>
       </c>
       <c r="G258" t="n">
         <v>64723.83</v>
@@ -7731,7 +7731,7 @@
         <v>661</v>
       </c>
       <c r="F261" t="n">
-        <v>247958</v>
+        <v>247955</v>
       </c>
       <c r="G261" t="n">
         <v>4064.4</v>
@@ -8207,7 +8207,7 @@
         <v>6</v>
       </c>
       <c r="F278" t="n">
-        <v>2308</v>
+        <v>2307</v>
       </c>
       <c r="G278" t="n">
         <v>0</v>
@@ -8266,10 +8266,10 @@
         <v>43821</v>
       </c>
       <c r="G280" t="n">
-        <v>38425.42</v>
+        <v>29951.69</v>
       </c>
       <c r="H280" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="281">
@@ -8291,7 +8291,7 @@
         <v>717</v>
       </c>
       <c r="F281" t="n">
-        <v>67723</v>
+        <v>67722</v>
       </c>
       <c r="G281" t="n">
         <v>43132.17</v>
@@ -8431,7 +8431,7 @@
         <v>39</v>
       </c>
       <c r="F286" t="n">
-        <v>9654</v>
+        <v>9653</v>
       </c>
       <c r="G286" t="n">
         <v>9785.580000000002</v>
@@ -8459,7 +8459,7 @@
         <v>33</v>
       </c>
       <c r="F287" t="n">
-        <v>3100</v>
+        <v>3099</v>
       </c>
       <c r="G287" t="n">
         <v>2206.79</v>
@@ -8627,7 +8627,7 @@
         <v>79</v>
       </c>
       <c r="F293" t="n">
-        <v>13077</v>
+        <v>13076</v>
       </c>
       <c r="G293" t="n">
         <v>11437.29</v>
@@ -9075,7 +9075,7 @@
         <v>235</v>
       </c>
       <c r="F309" t="n">
-        <v>18385</v>
+        <v>18384</v>
       </c>
       <c r="G309" t="n">
         <v>5647.48</v>
@@ -9187,7 +9187,7 @@
         <v>4</v>
       </c>
       <c r="F313" t="n">
-        <v>1442</v>
+        <v>1441</v>
       </c>
       <c r="G313" t="n">
         <v>0</v>
@@ -9243,7 +9243,7 @@
         <v>56</v>
       </c>
       <c r="F315" t="n">
-        <v>7278</v>
+        <v>7277</v>
       </c>
       <c r="G315" t="n">
         <v>5125.43</v>
@@ -9327,7 +9327,7 @@
         <v>31</v>
       </c>
       <c r="F318" t="n">
-        <v>3040</v>
+        <v>3039</v>
       </c>
       <c r="G318" t="n">
         <v>1439.84</v>
@@ -9355,7 +9355,7 @@
         <v>8</v>
       </c>
       <c r="F319" t="n">
-        <v>2047</v>
+        <v>2046</v>
       </c>
       <c r="G319" t="n">
         <v>0</v>
@@ -9495,7 +9495,7 @@
         <v>28</v>
       </c>
       <c r="F324" t="n">
-        <v>4407</v>
+        <v>4406</v>
       </c>
       <c r="G324" t="n">
         <v>0</v>
@@ -9523,7 +9523,7 @@
         <v>327</v>
       </c>
       <c r="F325" t="n">
-        <v>25587</v>
+        <v>25586</v>
       </c>
       <c r="G325" t="n">
         <v>16607.63</v>
@@ -9635,7 +9635,7 @@
         <v>7</v>
       </c>
       <c r="F329" t="n">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="G329" t="n">
         <v>1694.07</v>
@@ -9747,7 +9747,7 @@
         <v>18</v>
       </c>
       <c r="F333" t="n">
-        <v>2263</v>
+        <v>2262</v>
       </c>
       <c r="G333" t="n">
         <v>0</v>
@@ -9803,7 +9803,7 @@
         <v>216</v>
       </c>
       <c r="F335" t="n">
-        <v>21166</v>
+        <v>21165</v>
       </c>
       <c r="G335" t="n">
         <v>17370.34</v>
@@ -10083,7 +10083,7 @@
         <v>603</v>
       </c>
       <c r="F345" t="n">
-        <v>46410</v>
+        <v>46409</v>
       </c>
       <c r="G345" t="n">
         <v>21755.08</v>
@@ -10111,7 +10111,7 @@
         <v>181</v>
       </c>
       <c r="F346" t="n">
-        <v>12261</v>
+        <v>12260</v>
       </c>
       <c r="G346" t="n">
         <v>5507.63</v>
@@ -10226,10 +10226,10 @@
         <v>13490</v>
       </c>
       <c r="G350" t="n">
-        <v>20886.45</v>
+        <v>26224.59</v>
       </c>
       <c r="H350" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="351">
@@ -11343,7 +11343,7 @@
         <v>122</v>
       </c>
       <c r="F390" t="n">
-        <v>26170</v>
+        <v>26169</v>
       </c>
       <c r="G390" t="n">
         <v>0</v>
@@ -11654,10 +11654,10 @@
         <v>135452</v>
       </c>
       <c r="G8" t="n">
-        <v>4489.84</v>
+        <v>8556.790000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -12239,7 +12239,7 @@
         <v>976</v>
       </c>
       <c r="F29" t="n">
-        <v>229307</v>
+        <v>229304</v>
       </c>
       <c r="G29" t="n">
         <v>23462.71</v>
@@ -12569,13 +12569,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>7201.059999999999</v>
+        <v>7197.25</v>
       </c>
       <c r="E41" t="n">
-        <v>3478</v>
+        <v>3475</v>
       </c>
       <c r="F41" t="n">
-        <v>931242</v>
+        <v>931229</v>
       </c>
       <c r="G41" t="n">
         <v>27922.88</v>
@@ -12995,10 +12995,10 @@
         <v>3550.719946143185</v>
       </c>
       <c r="G6" t="n">
-        <v>18941.85973721108</v>
+        <v>21059.65973721108</v>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -13292,10 +13292,10 @@
         <v>3164.38</v>
       </c>
       <c r="G15" t="n">
-        <v>8005.1</v>
+        <v>10250.02</v>
       </c>
       <c r="H15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -13325,7 +13325,7 @@
         <v>1466.960624910898</v>
       </c>
       <c r="G16" t="n">
-        <v>10166.94</v>
+        <v>11558.23100175515</v>
       </c>
       <c r="H16" t="n">
         <v>3</v>
@@ -13391,10 +13391,10 @@
         <v>3178.5993750891</v>
       </c>
       <c r="G18" t="n">
-        <v>22029.65</v>
+        <v>25044.28899824484</v>
       </c>
       <c r="H18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(weekly-sync): auto-pull through 2026-06-23
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week25.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week25.xlsx
@@ -507,7 +507,7 @@
         <v>31</v>
       </c>
       <c r="F3" t="n">
-        <v>10166</v>
+        <v>10165</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -955,7 +955,7 @@
         <v>195</v>
       </c>
       <c r="F19" t="n">
-        <v>27760</v>
+        <v>27759</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1042,10 +1042,10 @@
         <v>18197</v>
       </c>
       <c r="G22" t="n">
-        <v>7033.05</v>
+        <v>12964.41</v>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -1319,7 +1319,7 @@
         <v>193</v>
       </c>
       <c r="F32" t="n">
-        <v>15482</v>
+        <v>15479</v>
       </c>
       <c r="G32" t="n">
         <v>14105.11</v>
@@ -1378,10 +1378,10 @@
         <v>21955</v>
       </c>
       <c r="G34" t="n">
-        <v>45803.08</v>
+        <v>48048</v>
       </c>
       <c r="H34" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="35">
@@ -1431,13 +1431,13 @@
         <v>1208</v>
       </c>
       <c r="F36" t="n">
-        <v>77503</v>
+        <v>77501</v>
       </c>
       <c r="G36" t="n">
-        <v>69973.03</v>
+        <v>72217.95</v>
       </c>
       <c r="H36" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="37">
@@ -1487,7 +1487,7 @@
         <v>70</v>
       </c>
       <c r="F38" t="n">
-        <v>17538</v>
+        <v>17537</v>
       </c>
       <c r="G38" t="n">
         <v>5464.42</v>
@@ -1882,10 +1882,10 @@
         <v>44439</v>
       </c>
       <c r="G52" t="n">
-        <v>60542.36</v>
+        <v>64609.3</v>
       </c>
       <c r="H52" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="53">
@@ -1935,13 +1935,13 @@
         <v>1047</v>
       </c>
       <c r="F54" t="n">
-        <v>124346</v>
+        <v>124345</v>
       </c>
       <c r="G54" t="n">
-        <v>64943.22</v>
+        <v>65366.1</v>
       </c>
       <c r="H54" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="55">
@@ -2019,7 +2019,7 @@
         <v>1099</v>
       </c>
       <c r="F57" t="n">
-        <v>182990</v>
+        <v>182987</v>
       </c>
       <c r="G57" t="n">
         <v>71935.60000000001</v>
@@ -2302,10 +2302,10 @@
         <v>8431</v>
       </c>
       <c r="G67" t="n">
-        <v>8811.860000000001</v>
+        <v>13217.79</v>
       </c>
       <c r="H67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="68">
@@ -2330,10 +2330,10 @@
         <v>2564</v>
       </c>
       <c r="G68" t="n">
-        <v>8811.860000000001</v>
+        <v>10209.32</v>
       </c>
       <c r="H68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="69">
@@ -2442,10 +2442,10 @@
         <v>66547</v>
       </c>
       <c r="G72" t="n">
-        <v>940.6799999999999</v>
+        <v>3566.95</v>
       </c>
       <c r="H72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73">
@@ -2610,10 +2610,10 @@
         <v>105674</v>
       </c>
       <c r="G78" t="n">
-        <v>85088.97</v>
+        <v>92715.24000000001</v>
       </c>
       <c r="H78" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="79">
@@ -2635,7 +2635,7 @@
         <v>832</v>
       </c>
       <c r="F79" t="n">
-        <v>172535</v>
+        <v>172534</v>
       </c>
       <c r="G79" t="n">
         <v>13251.67</v>
@@ -2803,7 +2803,7 @@
         <v>227</v>
       </c>
       <c r="F85" t="n">
-        <v>55144</v>
+        <v>55143</v>
       </c>
       <c r="G85" t="n">
         <v>4064.4</v>
@@ -2859,7 +2859,7 @@
         <v>16</v>
       </c>
       <c r="F87" t="n">
-        <v>2127</v>
+        <v>2126</v>
       </c>
       <c r="G87" t="n">
         <v>0</v>
@@ -3002,10 +3002,10 @@
         <v>103196</v>
       </c>
       <c r="G92" t="n">
-        <v>98942.53</v>
+        <v>106568.8</v>
       </c>
       <c r="H92" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="93">
@@ -3049,13 +3049,13 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>2569.55</v>
+        <v>2567.46</v>
       </c>
       <c r="E94" t="n">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F94" t="n">
-        <v>17095</v>
+        <v>17094</v>
       </c>
       <c r="G94" t="n">
         <v>19573.74</v>
@@ -3391,7 +3391,7 @@
         <v>35</v>
       </c>
       <c r="F106" t="n">
-        <v>5124</v>
+        <v>5121</v>
       </c>
       <c r="G106" t="n">
         <v>13131.35</v>
@@ -3419,7 +3419,7 @@
         <v>121</v>
       </c>
       <c r="F107" t="n">
-        <v>15334</v>
+        <v>15333</v>
       </c>
       <c r="G107" t="n">
         <v>7116.09</v>
@@ -3783,7 +3783,7 @@
         <v>28</v>
       </c>
       <c r="F120" t="n">
-        <v>11108</v>
+        <v>11106</v>
       </c>
       <c r="G120" t="n">
         <v>3219.49</v>
@@ -3923,7 +3923,7 @@
         <v>6</v>
       </c>
       <c r="F125" t="n">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="G125" t="n">
         <v>0</v>
@@ -3979,7 +3979,7 @@
         <v>19</v>
       </c>
       <c r="F127" t="n">
-        <v>4176</v>
+        <v>4175</v>
       </c>
       <c r="G127" t="n">
         <v>465.25</v>
@@ -4007,7 +4007,7 @@
         <v>3164</v>
       </c>
       <c r="F128" t="n">
-        <v>287082</v>
+        <v>287079</v>
       </c>
       <c r="G128" t="n">
         <v>13936.45</v>
@@ -4063,7 +4063,7 @@
         <v>32</v>
       </c>
       <c r="F130" t="n">
-        <v>6975</v>
+        <v>6974</v>
       </c>
       <c r="G130" t="n">
         <v>0</v>
@@ -4147,7 +4147,7 @@
         <v>889</v>
       </c>
       <c r="F133" t="n">
-        <v>152018</v>
+        <v>152016</v>
       </c>
       <c r="G133" t="n">
         <v>7412.71</v>
@@ -4175,7 +4175,7 @@
         <v>17</v>
       </c>
       <c r="F134" t="n">
-        <v>3294</v>
+        <v>3293</v>
       </c>
       <c r="G134" t="n">
         <v>0</v>
@@ -4287,13 +4287,13 @@
         <v>43</v>
       </c>
       <c r="F138" t="n">
-        <v>9818</v>
+        <v>9816</v>
       </c>
       <c r="G138" t="n">
-        <v>14022.02</v>
+        <v>17579.65</v>
       </c>
       <c r="H138" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="139">
@@ -4539,7 +4539,7 @@
         <v>183</v>
       </c>
       <c r="F147" t="n">
-        <v>39648</v>
+        <v>39647</v>
       </c>
       <c r="G147" t="n">
         <v>13217.79</v>
@@ -4595,7 +4595,7 @@
         <v>271</v>
       </c>
       <c r="F149" t="n">
-        <v>56809</v>
+        <v>56806</v>
       </c>
       <c r="G149" t="n">
         <v>5888.13</v>
@@ -4623,7 +4623,7 @@
         <v>175</v>
       </c>
       <c r="F150" t="n">
-        <v>29726</v>
+        <v>29725</v>
       </c>
       <c r="G150" t="n">
         <v>2389.83</v>
@@ -4791,7 +4791,7 @@
         <v>8</v>
       </c>
       <c r="F156" t="n">
-        <v>1858</v>
+        <v>1857</v>
       </c>
       <c r="G156" t="n">
         <v>0</v>
@@ -4987,7 +4987,7 @@
         <v>9</v>
       </c>
       <c r="F163" t="n">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="G163" t="n">
         <v>0</v>
@@ -5099,7 +5099,7 @@
         <v>614</v>
       </c>
       <c r="F167" t="n">
-        <v>149177</v>
+        <v>149174</v>
       </c>
       <c r="G167" t="n">
         <v>5122.87</v>
@@ -5127,7 +5127,7 @@
         <v>280</v>
       </c>
       <c r="F168" t="n">
-        <v>71610</v>
+        <v>71609</v>
       </c>
       <c r="G168" t="n">
         <v>8473.73</v>
@@ -5351,7 +5351,7 @@
         <v>318</v>
       </c>
       <c r="F176" t="n">
-        <v>51682</v>
+        <v>51681</v>
       </c>
       <c r="G176" t="n">
         <v>4913.56</v>
@@ -5547,7 +5547,7 @@
         <v>47</v>
       </c>
       <c r="F183" t="n">
-        <v>8163</v>
+        <v>8162</v>
       </c>
       <c r="G183" t="n">
         <v>0</v>
@@ -5575,7 +5575,7 @@
         <v>46</v>
       </c>
       <c r="F184" t="n">
-        <v>8029</v>
+        <v>8028</v>
       </c>
       <c r="G184" t="n">
         <v>1355.08</v>
@@ -5603,13 +5603,13 @@
         <v>272</v>
       </c>
       <c r="F185" t="n">
-        <v>31129</v>
+        <v>31128</v>
       </c>
       <c r="G185" t="n">
-        <v>17497.46</v>
+        <v>18683.05</v>
       </c>
       <c r="H185" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="186">
@@ -5687,7 +5687,7 @@
         <v>39</v>
       </c>
       <c r="F188" t="n">
-        <v>10713</v>
+        <v>10712</v>
       </c>
       <c r="G188" t="n">
         <v>1609.32</v>
@@ -5743,7 +5743,7 @@
         <v>108</v>
       </c>
       <c r="F190" t="n">
-        <v>18731</v>
+        <v>18730</v>
       </c>
       <c r="G190" t="n">
         <v>0</v>
@@ -5855,7 +5855,7 @@
         <v>2102</v>
       </c>
       <c r="F194" t="n">
-        <v>297709</v>
+        <v>297708</v>
       </c>
       <c r="G194" t="n">
         <v>13342.37</v>
@@ -6051,7 +6051,7 @@
         <v>3092</v>
       </c>
       <c r="F201" t="n">
-        <v>399975</v>
+        <v>399974</v>
       </c>
       <c r="G201" t="n">
         <v>19573.74</v>
@@ -6079,7 +6079,7 @@
         <v>576</v>
       </c>
       <c r="F202" t="n">
-        <v>69670</v>
+        <v>69669</v>
       </c>
       <c r="G202" t="n">
         <v>26314.41</v>
@@ -6275,7 +6275,7 @@
         <v>73</v>
       </c>
       <c r="F209" t="n">
-        <v>13095</v>
+        <v>13094</v>
       </c>
       <c r="G209" t="n">
         <v>15344.06</v>
@@ -6337,7 +6337,7 @@
         <v>22322.02</v>
       </c>
       <c r="H211" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="212">
@@ -6835,7 +6835,7 @@
         <v>14</v>
       </c>
       <c r="F229" t="n">
-        <v>2188</v>
+        <v>2187</v>
       </c>
       <c r="G229" t="n">
         <v>0</v>
@@ -7118,10 +7118,10 @@
         <v>4410</v>
       </c>
       <c r="G239" t="n">
-        <v>4744.06</v>
+        <v>6819.48</v>
       </c>
       <c r="H239" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="240">
@@ -7535,7 +7535,7 @@
         <v>68</v>
       </c>
       <c r="F254" t="n">
-        <v>7836</v>
+        <v>7835</v>
       </c>
       <c r="G254" t="n">
         <v>0</v>
@@ -7675,7 +7675,7 @@
         <v>148</v>
       </c>
       <c r="F259" t="n">
-        <v>10658</v>
+        <v>10656</v>
       </c>
       <c r="G259" t="n">
         <v>8135.550000000001</v>
@@ -7731,7 +7731,7 @@
         <v>661</v>
       </c>
       <c r="F261" t="n">
-        <v>247955</v>
+        <v>247954</v>
       </c>
       <c r="G261" t="n">
         <v>4064.4</v>
@@ -7759,7 +7759,7 @@
         <v>678</v>
       </c>
       <c r="F262" t="n">
-        <v>187082</v>
+        <v>187081</v>
       </c>
       <c r="G262" t="n">
         <v>8340.66</v>
@@ -8291,7 +8291,7 @@
         <v>717</v>
       </c>
       <c r="F281" t="n">
-        <v>67722</v>
+        <v>67720</v>
       </c>
       <c r="G281" t="n">
         <v>43132.17</v>
@@ -9775,7 +9775,7 @@
         <v>30</v>
       </c>
       <c r="F334" t="n">
-        <v>3971</v>
+        <v>3970</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
@@ -9797,13 +9797,13 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>1274.6</v>
+        <v>1272.58</v>
       </c>
       <c r="E335" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F335" t="n">
-        <v>21165</v>
+        <v>21163</v>
       </c>
       <c r="G335" t="n">
         <v>17370.34</v>
@@ -10055,7 +10055,7 @@
         <v>498</v>
       </c>
       <c r="F344" t="n">
-        <v>47333</v>
+        <v>47332</v>
       </c>
       <c r="G344" t="n">
         <v>5735.59</v>
@@ -10077,13 +10077,13 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>3036.37</v>
+        <v>3034.28</v>
       </c>
       <c r="E345" t="n">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="F345" t="n">
-        <v>46409</v>
+        <v>46408</v>
       </c>
       <c r="G345" t="n">
         <v>21755.08</v>
@@ -10117,7 +10117,7 @@
         <v>5507.63</v>
       </c>
       <c r="H346" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="347">
@@ -10643,13 +10643,13 @@
         <v>291</v>
       </c>
       <c r="F365" t="n">
-        <v>30904</v>
+        <v>30903</v>
       </c>
       <c r="G365" t="n">
         <v>7963.549999999999</v>
       </c>
       <c r="H365" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="366">
@@ -10811,7 +10811,7 @@
         <v>46</v>
       </c>
       <c r="F371" t="n">
-        <v>7495</v>
+        <v>7494</v>
       </c>
       <c r="G371" t="n">
         <v>0</v>
@@ -10895,7 +10895,7 @@
         <v>164</v>
       </c>
       <c r="F374" t="n">
-        <v>32658</v>
+        <v>32657</v>
       </c>
       <c r="G374" t="n">
         <v>6776.28</v>
@@ -10951,7 +10951,7 @@
         <v>80</v>
       </c>
       <c r="F376" t="n">
-        <v>10900</v>
+        <v>10898</v>
       </c>
       <c r="G376" t="n">
         <v>0</v>
@@ -11007,7 +11007,7 @@
         <v>10</v>
       </c>
       <c r="F378" t="n">
-        <v>6292</v>
+        <v>6291</v>
       </c>
       <c r="G378" t="n">
         <v>0</v>
@@ -11203,7 +11203,7 @@
         <v>42</v>
       </c>
       <c r="F385" t="n">
-        <v>8106</v>
+        <v>8105</v>
       </c>
       <c r="G385" t="n">
         <v>0</v>
@@ -11343,7 +11343,7 @@
         <v>122</v>
       </c>
       <c r="F390" t="n">
-        <v>26169</v>
+        <v>26168</v>
       </c>
       <c r="G390" t="n">
         <v>0</v>
@@ -11589,13 +11589,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6850.63</v>
+        <v>6848.15</v>
       </c>
       <c r="E6" t="n">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="F6" t="n">
-        <v>378402</v>
+        <v>378396</v>
       </c>
       <c r="G6" t="n">
         <v>16840.67</v>
@@ -11623,7 +11623,7 @@
         <v>278</v>
       </c>
       <c r="F7" t="n">
-        <v>65222</v>
+        <v>65217</v>
       </c>
       <c r="G7" t="n">
         <v>10164.42</v>
@@ -11654,10 +11654,10 @@
         <v>135452</v>
       </c>
       <c r="G8" t="n">
-        <v>8556.790000000001</v>
+        <v>4489.84</v>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -11822,10 +11822,10 @@
         <v>142678</v>
       </c>
       <c r="G14" t="n">
-        <v>25672.89</v>
+        <v>29739.84</v>
       </c>
       <c r="H14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15">
@@ -11875,7 +11875,7 @@
         <v>77</v>
       </c>
       <c r="F16" t="n">
-        <v>30853</v>
+        <v>30850</v>
       </c>
       <c r="G16" t="n">
         <v>2117.8</v>
@@ -12233,13 +12233,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2080.66</v>
+        <v>2079.44</v>
       </c>
       <c r="E29" t="n">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="F29" t="n">
-        <v>229304</v>
+        <v>229303</v>
       </c>
       <c r="G29" t="n">
         <v>23462.71</v>
@@ -12438,10 +12438,10 @@
         <v>148478</v>
       </c>
       <c r="G36" t="n">
-        <v>17594.9</v>
+        <v>19966.93</v>
       </c>
       <c r="H36" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37">
@@ -12569,13 +12569,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>7197.25</v>
+        <v>7192.37</v>
       </c>
       <c r="E41" t="n">
-        <v>3475</v>
+        <v>3471</v>
       </c>
       <c r="F41" t="n">
-        <v>931229</v>
+        <v>931226</v>
       </c>
       <c r="G41" t="n">
         <v>27922.88</v>
@@ -12718,10 +12718,10 @@
         <v>102076</v>
       </c>
       <c r="G46" t="n">
-        <v>11224.6</v>
+        <v>11732.23</v>
       </c>
       <c r="H46" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47">
@@ -12743,7 +12743,7 @@
         <v>2</v>
       </c>
       <c r="F47" t="n">
-        <v>1367</v>
+        <v>1366</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
@@ -12863,7 +12863,7 @@
         <v>2693.906634061338</v>
       </c>
       <c r="G2" t="n">
-        <v>5517.809999999999</v>
+        <v>5698.607558621674</v>
       </c>
       <c r="H2" t="n">
         <v>5</v>
@@ -12896,10 +12896,10 @@
         <v>3185.012276022305</v>
       </c>
       <c r="G3" t="n">
-        <v>6523.72</v>
+        <v>6737.47738728434</v>
       </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -12929,7 +12929,7 @@
         <v>2068.315839219331</v>
       </c>
       <c r="G4" t="n">
-        <v>4236.44</v>
+        <v>4375.251957868649</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
@@ -12962,7 +12962,7 @@
         <v>247.835250697026</v>
       </c>
       <c r="G5" t="n">
-        <v>507.63</v>
+        <v>524.263096225336</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>

</xml_diff>